<commit_message>
Correccion Excel Formato para deploy
</commit_message>
<xml_diff>
--- a/templates/excel/Nota.xlsx
+++ b/templates/excel/Nota.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/mauriciocv/Desktop/SS_Programs/SystemCrystal/BackendCrystal/templates/excel/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{33925EEA-28FA-A141-8215-3C6F93FEAD11}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{F683FE77-9C56-D046-805B-EA1A1D57CAF3}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="0" yWindow="780" windowWidth="24260" windowHeight="19500" tabRatio="663" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -830,75 +830,26 @@
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="0" fontId="14" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
+    <xf numFmtId="0" fontId="2" fillId="3" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="3" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="2" fillId="3" borderId="22" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="22" xfId="0" applyBorder="1"/>
+    <xf numFmtId="164" fontId="2" fillId="2" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="right" vertical="center"/>
+    </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="4" xfId="0" applyBorder="1"/>
-    <xf numFmtId="0" fontId="16" fillId="2" borderId="24" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="25" xfId="0" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="3" xfId="0" applyBorder="1"/>
-    <xf numFmtId="164" fontId="4" fillId="2" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="right" vertical="center"/>
-    </xf>
-    <xf numFmtId="164" fontId="9" fillId="3" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="right" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="13" fillId="3" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="9" fillId="3" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="2" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="20" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="20" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="2" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="13" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="12" fillId="3" borderId="31" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="11" xfId="0" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="14" xfId="0" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="16" xfId="0" applyBorder="1"/>
-    <xf numFmtId="165" fontId="2" fillId="2" borderId="3" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="165" fontId="2" fillId="2" borderId="3" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="15" fillId="3" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="5" xfId="0" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="6" xfId="0" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="7" xfId="0" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="8" xfId="0" applyBorder="1"/>
-    <xf numFmtId="164" fontId="8" fillId="3" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="right" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="13" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="3" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="3" borderId="32" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="23" xfId="0" applyBorder="1"/>
-    <xf numFmtId="164" fontId="2" fillId="2" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="right" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="18" fillId="2" borderId="12" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
-    <xf numFmtId="0" fontId="17" fillId="3" borderId="33" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" textRotation="255"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="12" xfId="0" applyBorder="1"/>
-    <xf numFmtId="0" fontId="2" fillId="3" borderId="22" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="22" xfId="0" applyBorder="1"/>
     <xf numFmtId="0" fontId="19" fillId="3" borderId="34" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
@@ -910,16 +861,65 @@
     <xf numFmtId="165" fontId="2" fillId="2" borderId="7" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="7" xfId="0" applyBorder="1"/>
     <xf numFmtId="16" fontId="13" fillId="3" borderId="22" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
+    <xf numFmtId="0" fontId="17" fillId="3" borderId="33" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" textRotation="255"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="12" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="14" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="18" fillId="2" borderId="12" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
+    <xf numFmtId="164" fontId="4" fillId="2" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="right" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="3" borderId="32" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="23" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="13" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="165" fontId="2" fillId="2" borderId="3" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
     <xf numFmtId="0" fontId="2" fillId="2" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="20" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="20" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="2" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center"/>
+    <xf numFmtId="0" fontId="13" fillId="3" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="3" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="13" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="12" fillId="3" borderId="31" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="11" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="16" xfId="0" applyBorder="1"/>
+    <xf numFmtId="165" fontId="2" fillId="2" borderId="3" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="15" fillId="3" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="5" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="6" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="8" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="16" fillId="2" borderId="24" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="25" xfId="0" applyBorder="1"/>
+    <xf numFmtId="164" fontId="9" fillId="3" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="right" vertical="center"/>
+    </xf>
+    <xf numFmtId="164" fontId="8" fillId="3" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="right" vertical="center"/>
     </xf>
   </cellXfs>
   <cellStyles count="2">
@@ -2074,72 +2074,72 @@
       <c r="A9" s="30" t="s">
         <v>4</v>
       </c>
-      <c r="B9" s="89"/>
-      <c r="C9" s="90"/>
-      <c r="D9" s="90"/>
-      <c r="E9" s="90"/>
+      <c r="B9" s="60"/>
+      <c r="C9" s="61"/>
+      <c r="D9" s="61"/>
+      <c r="E9" s="61"/>
       <c r="F9" s="48"/>
       <c r="G9" s="48" t="s">
         <v>5</v>
       </c>
       <c r="H9" s="48"/>
-      <c r="I9" s="98"/>
-      <c r="J9" s="90"/>
-      <c r="K9" s="90"/>
+      <c r="I9" s="76"/>
+      <c r="J9" s="61"/>
+      <c r="K9" s="61"/>
       <c r="L9" s="14"/>
     </row>
     <row r="10" spans="1:12" ht="13.5" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A10" s="30" t="s">
         <v>6</v>
       </c>
-      <c r="B10" s="81"/>
-      <c r="C10" s="61"/>
-      <c r="D10" s="61"/>
-      <c r="E10" s="61"/>
+      <c r="B10" s="58"/>
+      <c r="C10" s="59"/>
+      <c r="D10" s="59"/>
+      <c r="E10" s="59"/>
       <c r="F10" s="48"/>
       <c r="G10" s="48" t="s">
         <v>7</v>
       </c>
       <c r="H10" s="48"/>
-      <c r="I10" s="64"/>
-      <c r="J10" s="61"/>
-      <c r="K10" s="61"/>
+      <c r="I10" s="88"/>
+      <c r="J10" s="59"/>
+      <c r="K10" s="59"/>
       <c r="L10" s="14"/>
     </row>
     <row r="11" spans="1:12" ht="13.5" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A11" s="30" t="s">
         <v>8</v>
       </c>
-      <c r="B11" s="81"/>
-      <c r="C11" s="61"/>
-      <c r="D11" s="61"/>
-      <c r="E11" s="61"/>
+      <c r="B11" s="58"/>
+      <c r="C11" s="59"/>
+      <c r="D11" s="59"/>
+      <c r="E11" s="59"/>
       <c r="F11" s="48"/>
       <c r="G11" s="48" t="s">
         <v>9</v>
       </c>
       <c r="H11" s="48"/>
-      <c r="I11" s="99"/>
-      <c r="J11" s="61"/>
-      <c r="K11" s="61"/>
+      <c r="I11" s="87"/>
+      <c r="J11" s="59"/>
+      <c r="K11" s="59"/>
       <c r="L11" s="14"/>
     </row>
     <row r="12" spans="1:12" x14ac:dyDescent="0.15">
       <c r="A12" s="30" t="s">
         <v>10</v>
       </c>
-      <c r="B12" s="65"/>
-      <c r="C12" s="61"/>
-      <c r="D12" s="61"/>
-      <c r="E12" s="61"/>
+      <c r="B12" s="89"/>
+      <c r="C12" s="59"/>
+      <c r="D12" s="59"/>
+      <c r="E12" s="59"/>
       <c r="F12" s="48"/>
       <c r="G12" s="48" t="s">
         <v>11</v>
       </c>
       <c r="H12" s="48"/>
-      <c r="I12" s="73"/>
-      <c r="J12" s="61"/>
-      <c r="K12" s="61"/>
+      <c r="I12" s="94"/>
+      <c r="J12" s="59"/>
+      <c r="K12" s="59"/>
       <c r="L12" s="14"/>
     </row>
     <row r="13" spans="1:12" ht="6" customHeight="1" x14ac:dyDescent="0.15">
@@ -2174,43 +2174,43 @@
       <c r="A15" s="51" t="s">
         <v>12</v>
       </c>
-      <c r="B15" s="97"/>
-      <c r="C15" s="77"/>
-      <c r="D15" s="77"/>
+      <c r="B15" s="74"/>
+      <c r="C15" s="75"/>
+      <c r="D15" s="75"/>
       <c r="E15" s="32"/>
       <c r="F15" s="52"/>
-      <c r="G15" s="68" t="s">
+      <c r="G15" s="91" t="s">
         <v>13</v>
       </c>
-      <c r="H15" s="69"/>
-      <c r="I15" s="74"/>
-      <c r="J15" s="75"/>
-      <c r="K15" s="76"/>
+      <c r="H15" s="92"/>
+      <c r="I15" s="95"/>
+      <c r="J15" s="96"/>
+      <c r="K15" s="97"/>
       <c r="L15" s="10"/>
     </row>
     <row r="16" spans="1:12" ht="13.5" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A16" s="51" t="s">
         <v>14</v>
       </c>
-      <c r="B16" s="72"/>
-      <c r="C16" s="61"/>
-      <c r="D16" s="61"/>
+      <c r="B16" s="86"/>
+      <c r="C16" s="59"/>
+      <c r="D16" s="59"/>
       <c r="E16" s="32"/>
       <c r="F16" s="52"/>
-      <c r="G16" s="70"/>
-      <c r="H16" s="71"/>
-      <c r="I16" s="77"/>
-      <c r="J16" s="77"/>
-      <c r="K16" s="78"/>
+      <c r="G16" s="79"/>
+      <c r="H16" s="93"/>
+      <c r="I16" s="75"/>
+      <c r="J16" s="75"/>
+      <c r="K16" s="98"/>
       <c r="L16" s="10"/>
     </row>
     <row r="17" spans="1:12" x14ac:dyDescent="0.15">
       <c r="A17" s="51" t="s">
         <v>15</v>
       </c>
-      <c r="B17" s="72"/>
-      <c r="C17" s="61"/>
-      <c r="D17" s="61"/>
+      <c r="B17" s="86"/>
+      <c r="C17" s="59"/>
+      <c r="D17" s="59"/>
       <c r="E17" s="32"/>
       <c r="F17" s="52"/>
       <c r="G17" s="32"/>
@@ -2255,317 +2255,317 @@
       <c r="B20" s="56" t="s">
         <v>17</v>
       </c>
-      <c r="C20" s="80" t="s">
+      <c r="C20" s="85" t="s">
         <v>18</v>
       </c>
-      <c r="D20" s="61"/>
-      <c r="E20" s="61"/>
-      <c r="F20" s="58"/>
-      <c r="G20" s="67" t="s">
+      <c r="D20" s="59"/>
+      <c r="E20" s="59"/>
+      <c r="F20" s="63"/>
+      <c r="G20" s="90" t="s">
         <v>19</v>
       </c>
-      <c r="H20" s="58"/>
+      <c r="H20" s="63"/>
       <c r="I20" s="56" t="s">
         <v>20</v>
       </c>
-      <c r="J20" s="80" t="s">
+      <c r="J20" s="85" t="s">
         <v>21</v>
       </c>
-      <c r="K20" s="58"/>
+      <c r="K20" s="63"/>
       <c r="L20" s="15"/>
     </row>
     <row r="21" spans="1:12" x14ac:dyDescent="0.15">
       <c r="A21" s="17"/>
       <c r="B21" s="29"/>
-      <c r="C21" s="66"/>
-      <c r="D21" s="100"/>
-      <c r="E21" s="100"/>
-      <c r="F21" s="101"/>
-      <c r="G21" s="66"/>
-      <c r="H21" s="101"/>
+      <c r="C21" s="67"/>
+      <c r="D21" s="65"/>
+      <c r="E21" s="65"/>
+      <c r="F21" s="66"/>
+      <c r="G21" s="67"/>
+      <c r="H21" s="66"/>
       <c r="I21" s="1"/>
-      <c r="J21" s="84"/>
-      <c r="K21" s="101"/>
+      <c r="J21" s="62"/>
+      <c r="K21" s="66"/>
       <c r="L21" s="10"/>
     </row>
     <row r="22" spans="1:12" x14ac:dyDescent="0.15">
       <c r="A22" s="17"/>
       <c r="B22" s="29"/>
-      <c r="C22" s="66"/>
-      <c r="D22" s="100"/>
-      <c r="E22" s="100"/>
-      <c r="F22" s="101"/>
-      <c r="G22" s="66"/>
-      <c r="H22" s="101"/>
+      <c r="C22" s="67"/>
+      <c r="D22" s="65"/>
+      <c r="E22" s="65"/>
+      <c r="F22" s="66"/>
+      <c r="G22" s="67"/>
+      <c r="H22" s="66"/>
       <c r="I22" s="1"/>
-      <c r="J22" s="84"/>
-      <c r="K22" s="101"/>
+      <c r="J22" s="62"/>
+      <c r="K22" s="66"/>
       <c r="L22" s="10"/>
     </row>
     <row r="23" spans="1:12" x14ac:dyDescent="0.15">
       <c r="A23" s="17"/>
       <c r="B23" s="29"/>
-      <c r="C23" s="102"/>
-      <c r="D23" s="100"/>
-      <c r="E23" s="100"/>
-      <c r="F23" s="101"/>
-      <c r="G23" s="66"/>
-      <c r="H23" s="101"/>
+      <c r="C23" s="64"/>
+      <c r="D23" s="65"/>
+      <c r="E23" s="65"/>
+      <c r="F23" s="66"/>
+      <c r="G23" s="67"/>
+      <c r="H23" s="66"/>
       <c r="I23" s="1"/>
-      <c r="J23" s="84"/>
-      <c r="K23" s="101"/>
+      <c r="J23" s="62"/>
+      <c r="K23" s="66"/>
       <c r="L23" s="10"/>
     </row>
     <row r="24" spans="1:12" x14ac:dyDescent="0.15">
       <c r="A24" s="17"/>
       <c r="B24" s="29"/>
-      <c r="C24" s="102"/>
-      <c r="D24" s="100"/>
-      <c r="E24" s="100"/>
-      <c r="F24" s="101"/>
-      <c r="G24" s="66"/>
-      <c r="H24" s="101"/>
+      <c r="C24" s="64"/>
+      <c r="D24" s="65"/>
+      <c r="E24" s="65"/>
+      <c r="F24" s="66"/>
+      <c r="G24" s="67"/>
+      <c r="H24" s="66"/>
       <c r="I24" s="1"/>
-      <c r="J24" s="84"/>
-      <c r="K24" s="101"/>
+      <c r="J24" s="62"/>
+      <c r="K24" s="66"/>
       <c r="L24" s="10"/>
     </row>
     <row r="25" spans="1:12" x14ac:dyDescent="0.15">
       <c r="A25" s="17"/>
       <c r="B25" s="29"/>
-      <c r="C25" s="102"/>
-      <c r="D25" s="100"/>
-      <c r="E25" s="100"/>
-      <c r="F25" s="101"/>
-      <c r="G25" s="66"/>
-      <c r="H25" s="101"/>
+      <c r="C25" s="64"/>
+      <c r="D25" s="65"/>
+      <c r="E25" s="65"/>
+      <c r="F25" s="66"/>
+      <c r="G25" s="67"/>
+      <c r="H25" s="66"/>
       <c r="I25" s="1"/>
-      <c r="J25" s="84"/>
-      <c r="K25" s="101"/>
+      <c r="J25" s="62"/>
+      <c r="K25" s="66"/>
       <c r="L25" s="10"/>
     </row>
     <row r="26" spans="1:12" x14ac:dyDescent="0.15">
       <c r="A26" s="17"/>
       <c r="B26" s="29"/>
-      <c r="C26" s="102"/>
-      <c r="D26" s="100"/>
-      <c r="E26" s="100"/>
-      <c r="F26" s="101"/>
-      <c r="G26" s="66"/>
-      <c r="H26" s="101"/>
+      <c r="C26" s="64"/>
+      <c r="D26" s="65"/>
+      <c r="E26" s="65"/>
+      <c r="F26" s="66"/>
+      <c r="G26" s="67"/>
+      <c r="H26" s="66"/>
       <c r="I26" s="1"/>
-      <c r="J26" s="84"/>
-      <c r="K26" s="101"/>
+      <c r="J26" s="62"/>
+      <c r="K26" s="66"/>
       <c r="L26" s="10"/>
     </row>
     <row r="27" spans="1:12" x14ac:dyDescent="0.15">
       <c r="A27" s="17"/>
       <c r="B27" s="29"/>
-      <c r="C27" s="66"/>
-      <c r="D27" s="100"/>
-      <c r="E27" s="100"/>
-      <c r="F27" s="101"/>
-      <c r="G27" s="66"/>
-      <c r="H27" s="101"/>
+      <c r="C27" s="67"/>
+      <c r="D27" s="65"/>
+      <c r="E27" s="65"/>
+      <c r="F27" s="66"/>
+      <c r="G27" s="67"/>
+      <c r="H27" s="66"/>
       <c r="I27" s="1"/>
-      <c r="J27" s="84"/>
-      <c r="K27" s="101"/>
+      <c r="J27" s="62"/>
+      <c r="K27" s="66"/>
       <c r="L27" s="10"/>
     </row>
     <row r="28" spans="1:12" x14ac:dyDescent="0.15">
       <c r="A28" s="17"/>
       <c r="B28" s="29"/>
-      <c r="C28" s="66"/>
-      <c r="D28" s="100"/>
-      <c r="E28" s="100"/>
-      <c r="F28" s="101"/>
-      <c r="G28" s="66"/>
-      <c r="H28" s="101"/>
+      <c r="C28" s="67"/>
+      <c r="D28" s="65"/>
+      <c r="E28" s="65"/>
+      <c r="F28" s="66"/>
+      <c r="G28" s="67"/>
+      <c r="H28" s="66"/>
       <c r="I28" s="1"/>
-      <c r="J28" s="84"/>
-      <c r="K28" s="101"/>
+      <c r="J28" s="62"/>
+      <c r="K28" s="66"/>
       <c r="L28" s="10"/>
     </row>
     <row r="29" spans="1:12" x14ac:dyDescent="0.15">
       <c r="A29" s="17"/>
       <c r="B29" s="29"/>
-      <c r="C29" s="66"/>
-      <c r="D29" s="100"/>
-      <c r="E29" s="100"/>
-      <c r="F29" s="101"/>
-      <c r="G29" s="66"/>
-      <c r="H29" s="101"/>
+      <c r="C29" s="67"/>
+      <c r="D29" s="65"/>
+      <c r="E29" s="65"/>
+      <c r="F29" s="66"/>
+      <c r="G29" s="67"/>
+      <c r="H29" s="66"/>
       <c r="I29" s="1"/>
-      <c r="J29" s="84"/>
-      <c r="K29" s="101"/>
+      <c r="J29" s="62"/>
+      <c r="K29" s="66"/>
       <c r="L29" s="10"/>
     </row>
     <row r="30" spans="1:12" x14ac:dyDescent="0.15">
       <c r="A30" s="17"/>
       <c r="B30" s="29"/>
-      <c r="C30" s="66"/>
-      <c r="D30" s="100"/>
-      <c r="E30" s="100"/>
-      <c r="F30" s="101"/>
-      <c r="G30" s="66"/>
-      <c r="H30" s="101"/>
+      <c r="C30" s="67"/>
+      <c r="D30" s="65"/>
+      <c r="E30" s="65"/>
+      <c r="F30" s="66"/>
+      <c r="G30" s="67"/>
+      <c r="H30" s="66"/>
       <c r="I30" s="1"/>
-      <c r="J30" s="84"/>
-      <c r="K30" s="101"/>
+      <c r="J30" s="62"/>
+      <c r="K30" s="66"/>
       <c r="L30" s="10"/>
     </row>
     <row r="31" spans="1:12" x14ac:dyDescent="0.15">
       <c r="A31" s="17"/>
       <c r="B31" s="29"/>
-      <c r="C31" s="66"/>
-      <c r="D31" s="100"/>
-      <c r="E31" s="100"/>
-      <c r="F31" s="101"/>
-      <c r="G31" s="66"/>
-      <c r="H31" s="101"/>
+      <c r="C31" s="67"/>
+      <c r="D31" s="65"/>
+      <c r="E31" s="65"/>
+      <c r="F31" s="66"/>
+      <c r="G31" s="67"/>
+      <c r="H31" s="66"/>
       <c r="I31" s="1"/>
-      <c r="J31" s="84"/>
-      <c r="K31" s="101"/>
+      <c r="J31" s="62"/>
+      <c r="K31" s="66"/>
       <c r="L31" s="10"/>
     </row>
     <row r="32" spans="1:12" x14ac:dyDescent="0.15">
       <c r="A32" s="17"/>
       <c r="B32" s="29"/>
-      <c r="C32" s="66"/>
-      <c r="D32" s="100"/>
-      <c r="E32" s="100"/>
-      <c r="F32" s="101"/>
-      <c r="G32" s="66"/>
-      <c r="H32" s="101"/>
+      <c r="C32" s="67"/>
+      <c r="D32" s="65"/>
+      <c r="E32" s="65"/>
+      <c r="F32" s="66"/>
+      <c r="G32" s="67"/>
+      <c r="H32" s="66"/>
       <c r="I32" s="1"/>
-      <c r="J32" s="84"/>
-      <c r="K32" s="101"/>
+      <c r="J32" s="62"/>
+      <c r="K32" s="66"/>
       <c r="L32" s="10"/>
     </row>
     <row r="33" spans="1:12" x14ac:dyDescent="0.15">
       <c r="A33" s="17"/>
       <c r="B33" s="29"/>
-      <c r="C33" s="66"/>
-      <c r="D33" s="100"/>
-      <c r="E33" s="100"/>
-      <c r="F33" s="101"/>
-      <c r="G33" s="66"/>
-      <c r="H33" s="101"/>
+      <c r="C33" s="67"/>
+      <c r="D33" s="65"/>
+      <c r="E33" s="65"/>
+      <c r="F33" s="66"/>
+      <c r="G33" s="67"/>
+      <c r="H33" s="66"/>
       <c r="I33" s="1"/>
-      <c r="J33" s="84"/>
-      <c r="K33" s="101"/>
+      <c r="J33" s="62"/>
+      <c r="K33" s="66"/>
       <c r="L33" s="10"/>
     </row>
     <row r="34" spans="1:12" x14ac:dyDescent="0.15">
       <c r="A34" s="17"/>
       <c r="B34" s="29"/>
-      <c r="C34" s="66"/>
-      <c r="D34" s="100"/>
-      <c r="E34" s="100"/>
-      <c r="F34" s="101"/>
-      <c r="G34" s="66"/>
-      <c r="H34" s="101"/>
+      <c r="C34" s="67"/>
+      <c r="D34" s="65"/>
+      <c r="E34" s="65"/>
+      <c r="F34" s="66"/>
+      <c r="G34" s="67"/>
+      <c r="H34" s="66"/>
       <c r="I34" s="1"/>
-      <c r="J34" s="84"/>
-      <c r="K34" s="101"/>
+      <c r="J34" s="62"/>
+      <c r="K34" s="66"/>
       <c r="L34" s="10"/>
     </row>
     <row r="35" spans="1:12" x14ac:dyDescent="0.15">
       <c r="A35" s="17"/>
       <c r="B35" s="29"/>
-      <c r="C35" s="66"/>
-      <c r="D35" s="100"/>
-      <c r="E35" s="100"/>
-      <c r="F35" s="101"/>
-      <c r="G35" s="66"/>
-      <c r="H35" s="101"/>
+      <c r="C35" s="67"/>
+      <c r="D35" s="65"/>
+      <c r="E35" s="65"/>
+      <c r="F35" s="66"/>
+      <c r="G35" s="67"/>
+      <c r="H35" s="66"/>
       <c r="I35" s="1"/>
-      <c r="J35" s="84"/>
-      <c r="K35" s="101"/>
+      <c r="J35" s="62"/>
+      <c r="K35" s="66"/>
       <c r="L35" s="10"/>
     </row>
     <row r="36" spans="1:12" x14ac:dyDescent="0.15">
       <c r="A36" s="17"/>
       <c r="B36" s="29"/>
-      <c r="C36" s="66"/>
-      <c r="D36" s="100"/>
-      <c r="E36" s="100"/>
-      <c r="F36" s="101"/>
-      <c r="G36" s="66"/>
-      <c r="H36" s="101"/>
+      <c r="C36" s="67"/>
+      <c r="D36" s="65"/>
+      <c r="E36" s="65"/>
+      <c r="F36" s="66"/>
+      <c r="G36" s="67"/>
+      <c r="H36" s="66"/>
       <c r="I36" s="1"/>
-      <c r="J36" s="84"/>
-      <c r="K36" s="101"/>
+      <c r="J36" s="62"/>
+      <c r="K36" s="66"/>
       <c r="L36" s="10"/>
     </row>
     <row r="37" spans="1:12" x14ac:dyDescent="0.15">
       <c r="A37" s="17"/>
       <c r="B37" s="29"/>
-      <c r="C37" s="66"/>
-      <c r="D37" s="100"/>
-      <c r="E37" s="100"/>
-      <c r="F37" s="101"/>
-      <c r="G37" s="66"/>
-      <c r="H37" s="101"/>
+      <c r="C37" s="67"/>
+      <c r="D37" s="65"/>
+      <c r="E37" s="65"/>
+      <c r="F37" s="66"/>
+      <c r="G37" s="67"/>
+      <c r="H37" s="66"/>
       <c r="I37" s="1"/>
-      <c r="J37" s="84"/>
-      <c r="K37" s="101"/>
+      <c r="J37" s="62"/>
+      <c r="K37" s="66"/>
       <c r="L37" s="10"/>
     </row>
     <row r="38" spans="1:12" x14ac:dyDescent="0.15">
       <c r="A38" s="17"/>
       <c r="B38" s="29"/>
-      <c r="C38" s="66"/>
-      <c r="D38" s="100"/>
-      <c r="E38" s="100"/>
-      <c r="F38" s="101"/>
-      <c r="G38" s="66"/>
-      <c r="H38" s="101"/>
+      <c r="C38" s="67"/>
+      <c r="D38" s="65"/>
+      <c r="E38" s="65"/>
+      <c r="F38" s="66"/>
+      <c r="G38" s="67"/>
+      <c r="H38" s="66"/>
       <c r="I38" s="1"/>
-      <c r="J38" s="84"/>
-      <c r="K38" s="101"/>
+      <c r="J38" s="62"/>
+      <c r="K38" s="66"/>
       <c r="L38" s="10"/>
     </row>
     <row r="39" spans="1:12" x14ac:dyDescent="0.15">
       <c r="A39" s="17"/>
       <c r="B39" s="29"/>
-      <c r="C39" s="66"/>
-      <c r="D39" s="100"/>
-      <c r="E39" s="100"/>
-      <c r="F39" s="101"/>
-      <c r="G39" s="66"/>
-      <c r="H39" s="101"/>
+      <c r="C39" s="67"/>
+      <c r="D39" s="65"/>
+      <c r="E39" s="65"/>
+      <c r="F39" s="66"/>
+      <c r="G39" s="67"/>
+      <c r="H39" s="66"/>
       <c r="I39" s="1"/>
-      <c r="J39" s="84"/>
-      <c r="K39" s="101"/>
+      <c r="J39" s="62"/>
+      <c r="K39" s="66"/>
       <c r="L39" s="10"/>
     </row>
     <row r="40" spans="1:12" x14ac:dyDescent="0.15">
       <c r="A40" s="17"/>
       <c r="B40" s="29"/>
-      <c r="C40" s="66"/>
-      <c r="D40" s="100"/>
-      <c r="E40" s="100"/>
-      <c r="F40" s="101"/>
-      <c r="G40" s="66"/>
-      <c r="H40" s="101"/>
+      <c r="C40" s="67"/>
+      <c r="D40" s="65"/>
+      <c r="E40" s="65"/>
+      <c r="F40" s="66"/>
+      <c r="G40" s="67"/>
+      <c r="H40" s="66"/>
       <c r="I40" s="1"/>
-      <c r="J40" s="84"/>
-      <c r="K40" s="101"/>
+      <c r="J40" s="62"/>
+      <c r="K40" s="66"/>
       <c r="L40" s="10"/>
     </row>
     <row r="41" spans="1:12" x14ac:dyDescent="0.15">
       <c r="A41" s="28"/>
       <c r="B41" s="29"/>
-      <c r="C41" s="66"/>
-      <c r="D41" s="100"/>
-      <c r="E41" s="100"/>
-      <c r="F41" s="101"/>
-      <c r="G41" s="66"/>
-      <c r="H41" s="101"/>
+      <c r="C41" s="67"/>
+      <c r="D41" s="65"/>
+      <c r="E41" s="65"/>
+      <c r="F41" s="66"/>
+      <c r="G41" s="67"/>
+      <c r="H41" s="66"/>
       <c r="I41" s="1"/>
-      <c r="J41" s="84"/>
-      <c r="K41" s="101"/>
+      <c r="J41" s="62"/>
+      <c r="K41" s="66"/>
       <c r="L41" s="10"/>
     </row>
     <row r="42" spans="1:12" ht="12" customHeight="1" x14ac:dyDescent="0.15">
@@ -2580,42 +2580,42 @@
       <c r="I42" s="4" t="s">
         <v>22</v>
       </c>
-      <c r="J42" s="84"/>
-      <c r="K42" s="58"/>
+      <c r="J42" s="62"/>
+      <c r="K42" s="63"/>
       <c r="L42" s="10"/>
     </row>
     <row r="43" spans="1:12" ht="12.75" customHeight="1" x14ac:dyDescent="0.15">
-      <c r="A43" s="82" t="s">
+      <c r="A43" s="83" t="s">
         <v>23</v>
       </c>
-      <c r="B43" s="91"/>
-      <c r="C43" s="92"/>
-      <c r="D43" s="92"/>
-      <c r="E43" s="92"/>
-      <c r="F43" s="92"/>
-      <c r="G43" s="93"/>
+      <c r="B43" s="68"/>
+      <c r="C43" s="69"/>
+      <c r="D43" s="69"/>
+      <c r="E43" s="69"/>
+      <c r="F43" s="69"/>
+      <c r="G43" s="70"/>
       <c r="H43" s="32"/>
       <c r="I43" s="4" t="s">
         <v>24</v>
       </c>
-      <c r="J43" s="84"/>
-      <c r="K43" s="58"/>
+      <c r="J43" s="62"/>
+      <c r="K43" s="63"/>
       <c r="L43" s="10"/>
     </row>
     <row r="44" spans="1:12" ht="9.75" customHeight="1" x14ac:dyDescent="0.15">
-      <c r="A44" s="83"/>
-      <c r="B44" s="94"/>
-      <c r="C44" s="95"/>
-      <c r="D44" s="95"/>
-      <c r="E44" s="95"/>
-      <c r="F44" s="95"/>
-      <c r="G44" s="96"/>
+      <c r="A44" s="84"/>
+      <c r="B44" s="71"/>
+      <c r="C44" s="72"/>
+      <c r="D44" s="72"/>
+      <c r="E44" s="72"/>
+      <c r="F44" s="72"/>
+      <c r="G44" s="73"/>
       <c r="H44" s="33"/>
       <c r="I44" s="4" t="s">
         <v>25</v>
       </c>
-      <c r="J44" s="84"/>
-      <c r="K44" s="58"/>
+      <c r="J44" s="62"/>
+      <c r="K44" s="63"/>
       <c r="L44" s="10"/>
     </row>
     <row r="45" spans="1:12" ht="10.5" customHeight="1" x14ac:dyDescent="0.15">
@@ -2632,8 +2632,8 @@
       <c r="I45" s="47" t="s">
         <v>27</v>
       </c>
-      <c r="J45" s="63"/>
-      <c r="K45" s="58"/>
+      <c r="J45" s="101"/>
+      <c r="K45" s="63"/>
       <c r="L45" s="10"/>
     </row>
     <row r="46" spans="1:12" ht="10.5" customHeight="1" x14ac:dyDescent="0.15">
@@ -2652,8 +2652,8 @@
       <c r="I46" s="4" t="s">
         <v>30</v>
       </c>
-      <c r="J46" s="84"/>
-      <c r="K46" s="58"/>
+      <c r="J46" s="62"/>
+      <c r="K46" s="63"/>
       <c r="L46" s="10"/>
     </row>
     <row r="47" spans="1:12" ht="10.5" customHeight="1" x14ac:dyDescent="0.15">
@@ -2668,8 +2668,8 @@
       <c r="I47" s="3" t="s">
         <v>31</v>
       </c>
-      <c r="J47" s="62"/>
-      <c r="K47" s="58"/>
+      <c r="J47" s="82"/>
+      <c r="K47" s="63"/>
       <c r="L47" s="10"/>
     </row>
     <row r="48" spans="1:12" ht="11.25" customHeight="1" x14ac:dyDescent="0.15">
@@ -2690,8 +2690,8 @@
       <c r="I48" s="4" t="s">
         <v>34</v>
       </c>
-      <c r="J48" s="84"/>
-      <c r="K48" s="58"/>
+      <c r="J48" s="62"/>
+      <c r="K48" s="63"/>
       <c r="L48" s="10"/>
     </row>
     <row r="49" spans="1:17" ht="11.25" customHeight="1" x14ac:dyDescent="0.15">
@@ -2706,8 +2706,8 @@
       <c r="I49" s="35" t="s">
         <v>35</v>
       </c>
-      <c r="J49" s="79"/>
-      <c r="K49" s="58"/>
+      <c r="J49" s="102"/>
+      <c r="K49" s="63"/>
       <c r="L49" s="10"/>
     </row>
     <row r="50" spans="1:17" ht="11.25" customHeight="1" x14ac:dyDescent="0.15">
@@ -2729,7 +2729,7 @@
       <c r="L50" s="10"/>
     </row>
     <row r="51" spans="1:17" ht="11.25" customHeight="1" x14ac:dyDescent="0.15">
-      <c r="A51" s="87" t="s">
+      <c r="A51" s="77" t="s">
         <v>38</v>
       </c>
       <c r="B51" s="19"/>
@@ -2745,7 +2745,7 @@
       <c r="L51" s="10"/>
     </row>
     <row r="52" spans="1:17" ht="11.25" customHeight="1" x14ac:dyDescent="0.15">
-      <c r="A52" s="88"/>
+      <c r="A52" s="78"/>
       <c r="B52" s="19"/>
       <c r="C52" s="19"/>
       <c r="D52" s="19"/>
@@ -2753,15 +2753,15 @@
       <c r="F52" s="19"/>
       <c r="G52" s="19"/>
       <c r="H52" s="19"/>
-      <c r="I52" s="85" t="s">
+      <c r="I52" s="80" t="s">
         <v>39</v>
       </c>
-      <c r="J52" s="86"/>
-      <c r="K52" s="86"/>
+      <c r="J52" s="81"/>
+      <c r="K52" s="81"/>
       <c r="L52" s="10"/>
     </row>
     <row r="53" spans="1:17" ht="11.25" customHeight="1" x14ac:dyDescent="0.15">
-      <c r="A53" s="88"/>
+      <c r="A53" s="78"/>
       <c r="B53" s="19"/>
       <c r="C53" s="19"/>
       <c r="D53" s="19"/>
@@ -2775,7 +2775,7 @@
       <c r="L53" s="10"/>
     </row>
     <row r="54" spans="1:17" ht="11.25" customHeight="1" x14ac:dyDescent="0.15">
-      <c r="A54" s="88"/>
+      <c r="A54" s="78"/>
       <c r="B54" s="19"/>
       <c r="C54" s="19"/>
       <c r="D54" s="19"/>
@@ -2789,7 +2789,7 @@
       <c r="L54" s="10"/>
     </row>
     <row r="55" spans="1:17" ht="11.25" customHeight="1" x14ac:dyDescent="0.15">
-      <c r="A55" s="88"/>
+      <c r="A55" s="78"/>
       <c r="B55" s="19"/>
       <c r="C55" s="19"/>
       <c r="D55" s="19"/>
@@ -2803,7 +2803,7 @@
       <c r="L55" s="10"/>
     </row>
     <row r="56" spans="1:17" ht="11.25" customHeight="1" x14ac:dyDescent="0.15">
-      <c r="A56" s="88"/>
+      <c r="A56" s="78"/>
       <c r="B56" s="19"/>
       <c r="C56" s="19"/>
       <c r="D56" s="19"/>
@@ -2817,7 +2817,7 @@
       <c r="L56" s="10"/>
     </row>
     <row r="57" spans="1:17" ht="11.25" customHeight="1" x14ac:dyDescent="0.15">
-      <c r="A57" s="88"/>
+      <c r="A57" s="78"/>
       <c r="B57" s="19"/>
       <c r="C57" s="19"/>
       <c r="D57" s="19"/>
@@ -2831,7 +2831,7 @@
       <c r="L57" s="10"/>
     </row>
     <row r="58" spans="1:17" ht="11.25" customHeight="1" x14ac:dyDescent="0.15">
-      <c r="A58" s="88"/>
+      <c r="A58" s="78"/>
       <c r="B58" s="19"/>
       <c r="C58" s="19"/>
       <c r="D58" s="19"/>
@@ -2846,7 +2846,7 @@
       <c r="Q58" s="22"/>
     </row>
     <row r="59" spans="1:17" ht="11.25" customHeight="1" x14ac:dyDescent="0.15">
-      <c r="A59" s="88"/>
+      <c r="A59" s="78"/>
       <c r="B59" s="19"/>
       <c r="C59" s="19"/>
       <c r="D59" s="19"/>
@@ -2860,7 +2860,7 @@
       <c r="L59" s="10"/>
     </row>
     <row r="60" spans="1:17" ht="16.25" customHeight="1" x14ac:dyDescent="0.15">
-      <c r="A60" s="88"/>
+      <c r="A60" s="78"/>
       <c r="B60" s="19"/>
       <c r="C60" s="19"/>
       <c r="D60" s="19"/>
@@ -2874,7 +2874,7 @@
       <c r="L60" s="10"/>
     </row>
     <row r="61" spans="1:17" x14ac:dyDescent="0.15">
-      <c r="A61" s="88"/>
+      <c r="A61" s="78"/>
       <c r="B61" s="19"/>
       <c r="C61" s="19"/>
       <c r="D61" s="19"/>
@@ -2887,7 +2887,7 @@
       <c r="L61" s="10"/>
     </row>
     <row r="62" spans="1:17" x14ac:dyDescent="0.15">
-      <c r="A62" s="88"/>
+      <c r="A62" s="78"/>
       <c r="B62" s="19"/>
       <c r="C62" s="19"/>
       <c r="D62" s="19"/>
@@ -2900,7 +2900,7 @@
       <c r="L62" s="10"/>
     </row>
     <row r="63" spans="1:17" x14ac:dyDescent="0.15">
-      <c r="A63" s="88"/>
+      <c r="A63" s="78"/>
       <c r="B63" s="19"/>
       <c r="C63" s="19"/>
       <c r="D63" s="19"/>
@@ -2913,7 +2913,7 @@
       <c r="L63" s="10"/>
     </row>
     <row r="64" spans="1:17" x14ac:dyDescent="0.15">
-      <c r="A64" s="88"/>
+      <c r="A64" s="78"/>
       <c r="B64" s="19"/>
       <c r="C64" s="19"/>
       <c r="D64" s="19"/>
@@ -2925,7 +2925,7 @@
       <c r="L64" s="10"/>
     </row>
     <row r="65" spans="1:12" x14ac:dyDescent="0.15">
-      <c r="A65" s="88"/>
+      <c r="A65" s="78"/>
       <c r="B65" s="19"/>
       <c r="C65" s="19"/>
       <c r="D65" s="19"/>
@@ -2937,7 +2937,7 @@
       <c r="L65" s="10"/>
     </row>
     <row r="66" spans="1:12" x14ac:dyDescent="0.15">
-      <c r="A66" s="70"/>
+      <c r="A66" s="79"/>
       <c r="B66" s="19"/>
       <c r="C66" s="19"/>
       <c r="D66" s="19"/>
@@ -2998,15 +2998,91 @@
       <c r="F72" s="12"/>
       <c r="G72" s="12"/>
       <c r="H72" s="12"/>
-      <c r="I72" s="59" t="s">
+      <c r="I72" s="99" t="s">
         <v>40</v>
       </c>
-      <c r="J72" s="60"/>
-      <c r="K72" s="60"/>
+      <c r="J72" s="100"/>
+      <c r="K72" s="100"/>
       <c r="L72" s="13"/>
     </row>
   </sheetData>
   <mergeCells count="92">
+    <mergeCell ref="I72:K72"/>
+    <mergeCell ref="C39:F39"/>
+    <mergeCell ref="G23:H23"/>
+    <mergeCell ref="J28:K28"/>
+    <mergeCell ref="C32:F32"/>
+    <mergeCell ref="C37:F37"/>
+    <mergeCell ref="J45:K45"/>
+    <mergeCell ref="C24:F24"/>
+    <mergeCell ref="G34:H34"/>
+    <mergeCell ref="J34:K34"/>
+    <mergeCell ref="G38:H38"/>
+    <mergeCell ref="C30:F30"/>
+    <mergeCell ref="J49:K49"/>
+    <mergeCell ref="J27:K27"/>
+    <mergeCell ref="J36:K36"/>
+    <mergeCell ref="I10:K10"/>
+    <mergeCell ref="B12:E12"/>
+    <mergeCell ref="C26:F26"/>
+    <mergeCell ref="J31:K31"/>
+    <mergeCell ref="C41:F41"/>
+    <mergeCell ref="G20:H20"/>
+    <mergeCell ref="J21:K21"/>
+    <mergeCell ref="G22:H22"/>
+    <mergeCell ref="J23:K23"/>
+    <mergeCell ref="C27:F27"/>
+    <mergeCell ref="C36:F36"/>
+    <mergeCell ref="G15:H16"/>
+    <mergeCell ref="B17:D17"/>
+    <mergeCell ref="I12:K12"/>
+    <mergeCell ref="C28:F28"/>
+    <mergeCell ref="I15:K16"/>
+    <mergeCell ref="B11:E11"/>
+    <mergeCell ref="J22:K22"/>
+    <mergeCell ref="G26:H26"/>
+    <mergeCell ref="C20:F20"/>
+    <mergeCell ref="C21:F21"/>
+    <mergeCell ref="B16:D16"/>
+    <mergeCell ref="I11:K11"/>
+    <mergeCell ref="G21:H21"/>
+    <mergeCell ref="A43:A44"/>
+    <mergeCell ref="J46:K46"/>
+    <mergeCell ref="G25:H25"/>
+    <mergeCell ref="J20:K20"/>
+    <mergeCell ref="G24:H24"/>
+    <mergeCell ref="G33:H33"/>
+    <mergeCell ref="J47:K47"/>
+    <mergeCell ref="J43:K43"/>
+    <mergeCell ref="J33:K33"/>
+    <mergeCell ref="J48:K48"/>
+    <mergeCell ref="J29:K29"/>
+    <mergeCell ref="J38:K38"/>
+    <mergeCell ref="J40:K40"/>
+    <mergeCell ref="J25:K25"/>
+    <mergeCell ref="C29:F29"/>
+    <mergeCell ref="J42:K42"/>
+    <mergeCell ref="J39:K39"/>
+    <mergeCell ref="J41:K41"/>
+    <mergeCell ref="G39:H39"/>
+    <mergeCell ref="G35:H35"/>
+    <mergeCell ref="C40:F40"/>
+    <mergeCell ref="I9:K9"/>
+    <mergeCell ref="A51:A66"/>
+    <mergeCell ref="C22:F22"/>
+    <mergeCell ref="C31:F31"/>
+    <mergeCell ref="G32:H32"/>
+    <mergeCell ref="G41:H41"/>
+    <mergeCell ref="C25:F25"/>
+    <mergeCell ref="G29:H29"/>
+    <mergeCell ref="G31:H31"/>
+    <mergeCell ref="G40:H40"/>
+    <mergeCell ref="I52:K52"/>
+    <mergeCell ref="J24:K24"/>
+    <mergeCell ref="C34:F34"/>
+    <mergeCell ref="G37:H37"/>
+    <mergeCell ref="J26:K26"/>
+    <mergeCell ref="J35:K35"/>
     <mergeCell ref="B10:E10"/>
     <mergeCell ref="B9:E9"/>
     <mergeCell ref="J44:K44"/>
@@ -3023,82 +3099,6 @@
     <mergeCell ref="G30:H30"/>
     <mergeCell ref="C35:F35"/>
     <mergeCell ref="J32:K32"/>
-    <mergeCell ref="I9:K9"/>
-    <mergeCell ref="A51:A66"/>
-    <mergeCell ref="C22:F22"/>
-    <mergeCell ref="C31:F31"/>
-    <mergeCell ref="G32:H32"/>
-    <mergeCell ref="G41:H41"/>
-    <mergeCell ref="C25:F25"/>
-    <mergeCell ref="G29:H29"/>
-    <mergeCell ref="G31:H31"/>
-    <mergeCell ref="G40:H40"/>
-    <mergeCell ref="I52:K52"/>
-    <mergeCell ref="J24:K24"/>
-    <mergeCell ref="C34:F34"/>
-    <mergeCell ref="G37:H37"/>
-    <mergeCell ref="J26:K26"/>
-    <mergeCell ref="J35:K35"/>
-    <mergeCell ref="J25:K25"/>
-    <mergeCell ref="C29:F29"/>
-    <mergeCell ref="J42:K42"/>
-    <mergeCell ref="J39:K39"/>
-    <mergeCell ref="J41:K41"/>
-    <mergeCell ref="J47:K47"/>
-    <mergeCell ref="J43:K43"/>
-    <mergeCell ref="J33:K33"/>
-    <mergeCell ref="J48:K48"/>
-    <mergeCell ref="J29:K29"/>
-    <mergeCell ref="J38:K38"/>
-    <mergeCell ref="J40:K40"/>
-    <mergeCell ref="G39:H39"/>
-    <mergeCell ref="G35:H35"/>
-    <mergeCell ref="C40:F40"/>
-    <mergeCell ref="A43:A44"/>
-    <mergeCell ref="J46:K46"/>
-    <mergeCell ref="G25:H25"/>
-    <mergeCell ref="J20:K20"/>
-    <mergeCell ref="G24:H24"/>
-    <mergeCell ref="G33:H33"/>
-    <mergeCell ref="B11:E11"/>
-    <mergeCell ref="J22:K22"/>
-    <mergeCell ref="G26:H26"/>
-    <mergeCell ref="C20:F20"/>
-    <mergeCell ref="C21:F21"/>
-    <mergeCell ref="B16:D16"/>
-    <mergeCell ref="I11:K11"/>
-    <mergeCell ref="I10:K10"/>
-    <mergeCell ref="B12:E12"/>
-    <mergeCell ref="C26:F26"/>
-    <mergeCell ref="J31:K31"/>
-    <mergeCell ref="C41:F41"/>
-    <mergeCell ref="G20:H20"/>
-    <mergeCell ref="J21:K21"/>
-    <mergeCell ref="G22:H22"/>
-    <mergeCell ref="J23:K23"/>
-    <mergeCell ref="C27:F27"/>
-    <mergeCell ref="C36:F36"/>
-    <mergeCell ref="G15:H16"/>
-    <mergeCell ref="B17:D17"/>
-    <mergeCell ref="I12:K12"/>
-    <mergeCell ref="C28:F28"/>
-    <mergeCell ref="I15:K16"/>
-    <mergeCell ref="G21:H21"/>
-    <mergeCell ref="I72:K72"/>
-    <mergeCell ref="C39:F39"/>
-    <mergeCell ref="G23:H23"/>
-    <mergeCell ref="J28:K28"/>
-    <mergeCell ref="C32:F32"/>
-    <mergeCell ref="C37:F37"/>
-    <mergeCell ref="J45:K45"/>
-    <mergeCell ref="C24:F24"/>
-    <mergeCell ref="G34:H34"/>
-    <mergeCell ref="J34:K34"/>
-    <mergeCell ref="G38:H38"/>
-    <mergeCell ref="C30:F30"/>
-    <mergeCell ref="J49:K49"/>
-    <mergeCell ref="J27:K27"/>
-    <mergeCell ref="J36:K36"/>
   </mergeCells>
   <pageMargins left="0.25" right="0.25" top="0.25" bottom="0.25" header="0.16669999999999999" footer="0.16669999999999999"/>
   <pageSetup paperSize="9" orientation="portrait" horizontalDpi="0" verticalDpi="0"/>

</xml_diff>